<commit_message>
implemented topN for mixed
</commit_message>
<xml_diff>
--- a/owlcms/src/main/resources/templates/teamResults/TeamResults-A4.xlsx
+++ b/owlcms/src/main/resources/templates/teamResults/TeamResults-A4.xlsx
@@ -56,7 +56,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>jx:each(items="team.sortedTeamMembers" var="member" lastCell="G5")</t>
+          <t>jx:each(items="team.countedTeamMembers" var="member" lastCell="G5")</t>
         </r>
       </text>
     </comment>
@@ -105,7 +105,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>jx:each(items="team.sortedTeamMembers" var="member" lastCell="G5")</t>
+          <t>jx:each(items="team.countedTeamMembers" var="member" lastCell="G5")</t>
         </r>
       </text>
     </comment>
@@ -154,7 +154,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>jx:each(items="team.sortedTeamMembers" var="member" lastCell="G5")</t>
+          <t>jx:each(items="team.countedTeamMembers" var="member" lastCell="G5")</t>
         </r>
       </text>
     </comment>
@@ -163,7 +163,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="29">
   <si>
     <t>${competition.competitionName}</t>
   </si>
@@ -180,7 +180,7 @@
     <t>${mShowPoints &amp;&amp; team.points != 0 ? team.points : ""}</t>
   </si>
   <si>
-    <t>${team.counted}/${team.size}</t>
+    <t>${team.counted}/${mTeamSize != 0 ? mTeamSize : team.size}</t>
   </si>
   <si>
     <t>${!mShowPoints &amp;&amp; team.score != 0 ? team.score : ""}</t>
@@ -228,6 +228,9 @@
     <t>${wShowPoints &amp;&amp; team.points != 0 ? team.points : ""}</t>
   </si>
   <si>
+    <t>${team.counted}/${wTeamSize != 0 ? wTeamSize : team.size}</t>
+  </si>
+  <si>
     <t>${!wShowPoints &amp;&amp; team.score != 0 ? team.score : ""}</t>
   </si>
   <si>
@@ -238,6 +241,9 @@
   </si>
   <si>
     <t>${mwShowPoints &amp;&amp; team.points != 0 ? team.points : ""}</t>
+  </si>
+  <si>
+    <t>${team.counted}/${mwTeamSize != 0 ? mwTeamSize : team.size}</t>
   </si>
   <si>
     <t>${!mwShowPoints &amp;&amp; team.score != 0 ? team.score : ""}</t>
@@ -783,10 +789,10 @@
         <v>20</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -807,7 +813,7 @@
         <v>11</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -865,7 +871,7 @@
         <v>1</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -876,13 +882,13 @@
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
       <c r="E3" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -903,7 +909,7 @@
         <v>11</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:7">

</xml_diff>